<commit_message>
Apply OVE corporate Excel format
</commit_message>
<xml_diff>
--- a/assets/data/world-bank/catalog/catalogo_dataset_web_ove_banco_mundial.xlsx
+++ b/assets/data/world-bank/catalog/catalogo_dataset_web_ove_banco_mundial.xlsx
@@ -1,13 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="catalogo" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="catalogo" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="metadatos" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,7 +18,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="5">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -25,13 +26,35 @@
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="000A2D5A"/>
+      <sz val="14"/>
+    </font>
+    <font>
+      <color rgb="006B6B6B"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="000A2D5A"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="000A2D5A"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -46,82 +69,86 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <colors>
-    <indexedColors>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008000"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00808000"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="00C0C0C0"/>
-      <rgbColor rgb="00808080"/>
-      <rgbColor rgb="009999FF"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00FFFFCC"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00660066"/>
-      <rgbColor rgb="00FF8080"/>
-      <rgbColor rgb="000066CC"/>
-      <rgbColor rgb="00CCCCFF"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="0000CCFF"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00CCFFCC"/>
-      <rgbColor rgb="00FFFF99"/>
-      <rgbColor rgb="0099CCFF"/>
-      <rgbColor rgb="00FF99CC"/>
-      <rgbColor rgb="00CC99FF"/>
-      <rgbColor rgb="00FFCC99"/>
-      <rgbColor rgb="003366FF"/>
-      <rgbColor rgb="0033CCCC"/>
-      <rgbColor rgb="0099CC00"/>
-      <rgbColor rgb="00FFCC00"/>
-      <rgbColor rgb="00FF9900"/>
-      <rgbColor rgb="00FF6600"/>
-      <rgbColor rgb="00666699"/>
-      <rgbColor rgb="00969696"/>
-      <rgbColor rgb="00003366"/>
-      <rgbColor rgb="00339966"/>
-      <rgbColor rgb="00003300"/>
-      <rgbColor rgb="00333300"/>
-      <rgbColor rgb="00993300"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00333399"/>
-      <rgbColor rgb="00333333"/>
-    </indexedColors>
-  </colors>
 </styleSheet>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>0</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1809750" cy="457200"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="1" name="Image 1" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId1"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
+</file>
+
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>0</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1809750" cy="457200"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="1" name="Image 1" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId1"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -413,557 +440,587 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J13"/>
+  <dimension ref="A1:J18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="24" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="8" max="8"/>
+    <col width="18" customWidth="1" min="9" max="9"/>
+    <col width="18" customWidth="1" min="10" max="10"/>
+  </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
+    <row r="1" ht="28" customHeight="1">
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Catálogo Banco Mundial</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="22" customHeight="1">
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>Venezuela</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="18" customHeight="1"/>
+    <row r="4" ht="16" customHeight="1"/>
+    <row r="5" ht="8" customHeight="1"/>
+    <row r="6" ht="24" customHeight="1">
+      <c r="A6" s="3" t="inlineStr">
         <is>
           <t>Área temática</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B6" s="3" t="inlineStr">
         <is>
           <t>ID área</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C6" s="3" t="inlineStr">
         <is>
           <t>Registros</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D6" s="3" t="inlineStr">
         <is>
           <t>Indicadores</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E6" s="3" t="inlineStr">
         <is>
           <t>Primer año</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F6" s="3" t="inlineStr">
         <is>
           <t>Último año</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G6" s="3" t="inlineStr">
         <is>
           <t>Último año con dato</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H6" s="3" t="inlineStr">
         <is>
           <t>Archivo CSV</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I6" s="3" t="inlineStr">
         <is>
           <t>Archivo JSON</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J6" s="3" t="inlineStr">
         <is>
           <t>Archivo Excel</t>
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
         <is>
           <t>Demografía</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="B7" s="4" t="inlineStr">
         <is>
           <t>demografia</t>
         </is>
       </c>
-      <c r="C2" t="n">
+      <c r="C7" s="4" t="n">
         <v>528</v>
       </c>
-      <c r="D2" t="n">
+      <c r="D7" s="4" t="n">
         <v>8</v>
       </c>
-      <c r="E2" t="n">
+      <c r="E7" s="4" t="n">
         <v>1960</v>
       </c>
-      <c r="F2" t="n">
+      <c r="F7" s="4" t="n">
         <v>2025</v>
       </c>
-      <c r="G2" t="n">
+      <c r="G7" s="4" t="n">
         <v>2025</v>
       </c>
-      <c r="H2" t="inlineStr">
+      <c r="H7" s="4" t="inlineStr">
         <is>
           <t>assets/data/world-bank/csv/ove_banco_mundial_venezuela_demografia.csv</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr">
+      <c r="I7" s="4" t="inlineStr">
         <is>
           <t>assets/data/world-bank/json/ove_banco_mundial_venezuela_demografia.json</t>
         </is>
       </c>
-      <c r="J2" t="inlineStr">
+      <c r="J7" s="4" t="inlineStr">
         <is>
           <t>assets/data/world-bank/excel/ove_banco_mundial_venezuela_demografia.xlsx</t>
         </is>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
         <is>
           <t>Educación</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="B8" s="4" t="inlineStr">
         <is>
           <t>educacion</t>
         </is>
       </c>
-      <c r="C3" t="n">
+      <c r="C8" s="4" t="n">
         <v>333</v>
       </c>
-      <c r="D3" t="n">
+      <c r="D8" s="4" t="n">
         <v>5</v>
       </c>
-      <c r="E3" t="n">
+      <c r="E8" s="4" t="n">
         <v>1960</v>
       </c>
-      <c r="F3" t="n">
+      <c r="F8" s="4" t="n">
         <v>2026</v>
       </c>
-      <c r="G3" t="n">
+      <c r="G8" s="4" t="n">
         <v>2017</v>
       </c>
-      <c r="H3" t="inlineStr">
+      <c r="H8" s="4" t="inlineStr">
         <is>
           <t>assets/data/world-bank/csv/ove_banco_mundial_venezuela_educacion.csv</t>
         </is>
       </c>
-      <c r="I3" t="inlineStr">
+      <c r="I8" s="4" t="inlineStr">
         <is>
           <t>assets/data/world-bank/json/ove_banco_mundial_venezuela_educacion.json</t>
         </is>
       </c>
-      <c r="J3" t="inlineStr">
+      <c r="J8" s="4" t="inlineStr">
         <is>
           <t>assets/data/world-bank/excel/ove_banco_mundial_venezuela_educacion.xlsx</t>
         </is>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
         <is>
           <t>Energía y ambiente</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
+      <c r="B9" s="4" t="inlineStr">
         <is>
           <t>energia_y_ambiente</t>
         </is>
       </c>
-      <c r="C4" t="n">
+      <c r="C9" s="4" t="n">
         <v>334</v>
       </c>
-      <c r="D4" t="n">
+      <c r="D9" s="4" t="n">
         <v>5</v>
       </c>
-      <c r="E4" t="n">
+      <c r="E9" s="4" t="n">
         <v>1960</v>
       </c>
-      <c r="F4" t="n">
+      <c r="F9" s="4" t="n">
         <v>2026</v>
       </c>
-      <c r="G4" t="n">
+      <c r="G9" s="4" t="n">
         <v>2014</v>
       </c>
-      <c r="H4" t="inlineStr">
+      <c r="H9" s="4" t="inlineStr">
         <is>
           <t>assets/data/world-bank/csv/ove_banco_mundial_venezuela_energia_y_ambiente.csv</t>
         </is>
       </c>
-      <c r="I4" t="inlineStr">
+      <c r="I9" s="4" t="inlineStr">
         <is>
           <t>assets/data/world-bank/json/ove_banco_mundial_venezuela_energia_y_ambiente.json</t>
         </is>
       </c>
-      <c r="J4" t="inlineStr">
+      <c r="J9" s="4" t="inlineStr">
         <is>
           <t>assets/data/world-bank/excel/ove_banco_mundial_venezuela_energia_y_ambiente.xlsx</t>
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
         <is>
           <t>Género</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
+      <c r="B10" s="4" t="inlineStr">
         <is>
           <t>genero</t>
         </is>
       </c>
-      <c r="C5" t="n">
+      <c r="C10" s="4" t="n">
         <v>331</v>
       </c>
-      <c r="D5" t="n">
+      <c r="D10" s="4" t="n">
         <v>5</v>
       </c>
-      <c r="E5" t="n">
+      <c r="E10" s="4" t="n">
         <v>1960</v>
       </c>
-      <c r="F5" t="n">
+      <c r="F10" s="4" t="n">
         <v>2026</v>
       </c>
-      <c r="G5" t="n">
+      <c r="G10" s="4" t="n">
         <v>2025</v>
       </c>
-      <c r="H5" t="inlineStr">
+      <c r="H10" s="4" t="inlineStr">
         <is>
           <t>assets/data/world-bank/csv/ove_banco_mundial_venezuela_genero.csv</t>
         </is>
       </c>
-      <c r="I5" t="inlineStr">
+      <c r="I10" s="4" t="inlineStr">
         <is>
           <t>assets/data/world-bank/json/ove_banco_mundial_venezuela_genero.json</t>
         </is>
       </c>
-      <c r="J5" t="inlineStr">
+      <c r="J10" s="4" t="inlineStr">
         <is>
           <t>assets/data/world-bank/excel/ove_banco_mundial_venezuela_genero.xlsx</t>
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
         <is>
           <t>Infraestructura y digitalización</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr">
+      <c r="B11" s="4" t="inlineStr">
         <is>
           <t>infraestructura_y_digitalizacion</t>
         </is>
       </c>
-      <c r="C6" t="n">
+      <c r="C11" s="4" t="n">
         <v>264</v>
       </c>
-      <c r="D6" t="n">
+      <c r="D11" s="4" t="n">
         <v>4</v>
       </c>
-      <c r="E6" t="n">
+      <c r="E11" s="4" t="n">
         <v>1960</v>
       </c>
-      <c r="F6" t="n">
+      <c r="F11" s="4" t="n">
         <v>2025</v>
       </c>
-      <c r="G6" t="n">
+      <c r="G11" s="4" t="n">
         <v>2024</v>
       </c>
-      <c r="H6" t="inlineStr">
+      <c r="H11" s="4" t="inlineStr">
         <is>
           <t>assets/data/world-bank/csv/ove_banco_mundial_venezuela_infraestructura_y_digitalizacion.csv</t>
         </is>
       </c>
-      <c r="I6" t="inlineStr">
+      <c r="I11" s="4" t="inlineStr">
         <is>
           <t>assets/data/world-bank/json/ove_banco_mundial_venezuela_infraestructura_y_digitalizacion.json</t>
         </is>
       </c>
-      <c r="J6" t="inlineStr">
+      <c r="J11" s="4" t="inlineStr">
         <is>
           <t>assets/data/world-bank/excel/ove_banco_mundial_venezuela_infraestructura_y_digitalizacion.xlsx</t>
         </is>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
         <is>
           <t>Macroeconomía</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr">
+      <c r="B12" s="4" t="inlineStr">
         <is>
           <t>macroeconomia</t>
         </is>
       </c>
-      <c r="C7" t="n">
+      <c r="C12" s="4" t="n">
         <v>666</v>
       </c>
-      <c r="D7" t="n">
+      <c r="D12" s="4" t="n">
         <v>10</v>
       </c>
-      <c r="E7" t="n">
+      <c r="E12" s="4" t="n">
         <v>1960</v>
       </c>
-      <c r="F7" t="n">
+      <c r="F12" s="4" t="n">
         <v>2026</v>
       </c>
-      <c r="G7" t="n">
+      <c r="G12" s="4" t="n">
         <v>2025</v>
       </c>
-      <c r="H7" t="inlineStr">
+      <c r="H12" s="4" t="inlineStr">
         <is>
           <t>assets/data/world-bank/csv/ove_banco_mundial_venezuela_macroeconomia.csv</t>
         </is>
       </c>
-      <c r="I7" t="inlineStr">
+      <c r="I12" s="4" t="inlineStr">
         <is>
           <t>assets/data/world-bank/json/ove_banco_mundial_venezuela_macroeconomia.json</t>
         </is>
       </c>
-      <c r="J7" t="inlineStr">
+      <c r="J12" s="4" t="inlineStr">
         <is>
           <t>assets/data/world-bank/excel/ove_banco_mundial_venezuela_macroeconomia.xlsx</t>
         </is>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
         <is>
           <t>Mercado laboral</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr">
+      <c r="B13" s="4" t="inlineStr">
         <is>
           <t>mercado_laboral</t>
         </is>
       </c>
-      <c r="C8" t="n">
+      <c r="C13" s="4" t="n">
         <v>662</v>
       </c>
-      <c r="D8" t="n">
+      <c r="D13" s="4" t="n">
         <v>10</v>
       </c>
-      <c r="E8" t="n">
+      <c r="E13" s="4" t="n">
         <v>1960</v>
       </c>
-      <c r="F8" t="n">
+      <c r="F13" s="4" t="n">
         <v>2026</v>
       </c>
-      <c r="G8" t="n">
+      <c r="G13" s="4" t="n">
         <v>2025</v>
       </c>
-      <c r="H8" t="inlineStr">
+      <c r="H13" s="4" t="inlineStr">
         <is>
           <t>assets/data/world-bank/csv/ove_banco_mundial_venezuela_mercado_laboral.csv</t>
         </is>
       </c>
-      <c r="I8" t="inlineStr">
+      <c r="I13" s="4" t="inlineStr">
         <is>
           <t>assets/data/world-bank/json/ove_banco_mundial_venezuela_mercado_laboral.json</t>
         </is>
       </c>
-      <c r="J8" t="inlineStr">
+      <c r="J13" s="4" t="inlineStr">
         <is>
           <t>assets/data/world-bank/excel/ove_banco_mundial_venezuela_mercado_laboral.xlsx</t>
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
         <is>
           <t>Pobreza y desigualdad</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr">
+      <c r="B14" s="4" t="inlineStr">
         <is>
           <t>pobreza_y_desigualdad</t>
         </is>
       </c>
-      <c r="C9" t="n">
+      <c r="C14" s="4" t="n">
         <v>331</v>
       </c>
-      <c r="D9" t="n">
+      <c r="D14" s="4" t="n">
         <v>5</v>
       </c>
-      <c r="E9" t="n">
+      <c r="E14" s="4" t="n">
         <v>1960</v>
       </c>
-      <c r="F9" t="n">
+      <c r="F14" s="4" t="n">
         <v>2026</v>
       </c>
-      <c r="G9" t="n">
+      <c r="G14" s="4" t="n">
         <v>2015</v>
       </c>
-      <c r="H9" t="inlineStr">
+      <c r="H14" s="4" t="inlineStr">
         <is>
           <t>assets/data/world-bank/csv/ove_banco_mundial_venezuela_pobreza_y_desigualdad.csv</t>
         </is>
       </c>
-      <c r="I9" t="inlineStr">
+      <c r="I14" s="4" t="inlineStr">
         <is>
           <t>assets/data/world-bank/json/ove_banco_mundial_venezuela_pobreza_y_desigualdad.json</t>
         </is>
       </c>
-      <c r="J9" t="inlineStr">
+      <c r="J14" s="4" t="inlineStr">
         <is>
           <t>assets/data/world-bank/excel/ove_banco_mundial_venezuela_pobreza_y_desigualdad.xlsx</t>
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
         <is>
           <t>Precios e inflación</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr">
+      <c r="B15" s="4" t="inlineStr">
         <is>
           <t>precios_e_inflacion</t>
         </is>
       </c>
-      <c r="C10" t="n">
+      <c r="C15" s="4" t="n">
         <v>467</v>
       </c>
-      <c r="D10" t="n">
+      <c r="D15" s="4" t="n">
         <v>7</v>
       </c>
-      <c r="E10" t="n">
+      <c r="E15" s="4" t="n">
         <v>1960</v>
       </c>
-      <c r="F10" t="n">
+      <c r="F15" s="4" t="n">
         <v>2026</v>
       </c>
-      <c r="G10" t="n">
+      <c r="G15" s="4" t="n">
         <v>2025</v>
       </c>
-      <c r="H10" t="inlineStr">
+      <c r="H15" s="4" t="inlineStr">
         <is>
           <t>assets/data/world-bank/csv/ove_banco_mundial_venezuela_precios_e_inflacion.csv</t>
         </is>
       </c>
-      <c r="I10" t="inlineStr">
+      <c r="I15" s="4" t="inlineStr">
         <is>
           <t>assets/data/world-bank/json/ove_banco_mundial_venezuela_precios_e_inflacion.json</t>
         </is>
       </c>
-      <c r="J10" t="inlineStr">
+      <c r="J15" s="4" t="inlineStr">
         <is>
           <t>assets/data/world-bank/excel/ove_banco_mundial_venezuela_precios_e_inflacion.xlsx</t>
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
         <is>
           <t>Salud</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr">
+      <c r="B16" s="4" t="inlineStr">
         <is>
           <t>salud</t>
         </is>
       </c>
-      <c r="C11" t="n">
+      <c r="C16" s="4" t="n">
         <v>463</v>
       </c>
-      <c r="D11" t="n">
+      <c r="D16" s="4" t="n">
         <v>7</v>
       </c>
-      <c r="E11" t="n">
+      <c r="E16" s="4" t="n">
         <v>1960</v>
       </c>
-      <c r="F11" t="n">
+      <c r="F16" s="4" t="n">
         <v>2026</v>
       </c>
-      <c r="G11" t="n">
+      <c r="G16" s="4" t="n">
         <v>2024</v>
       </c>
-      <c r="H11" t="inlineStr">
+      <c r="H16" s="4" t="inlineStr">
         <is>
           <t>assets/data/world-bank/csv/ove_banco_mundial_venezuela_salud.csv</t>
         </is>
       </c>
-      <c r="I11" t="inlineStr">
+      <c r="I16" s="4" t="inlineStr">
         <is>
           <t>assets/data/world-bank/json/ove_banco_mundial_venezuela_salud.json</t>
         </is>
       </c>
-      <c r="J11" t="inlineStr">
+      <c r="J16" s="4" t="inlineStr">
         <is>
           <t>assets/data/world-bank/excel/ove_banco_mundial_venezuela_salud.xlsx</t>
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
         <is>
           <t>Sector externo</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr">
+      <c r="B17" s="4" t="inlineStr">
         <is>
           <t>sector_externo</t>
         </is>
       </c>
-      <c r="C12" t="n">
+      <c r="C17" s="4" t="n">
         <v>602</v>
       </c>
-      <c r="D12" t="n">
+      <c r="D17" s="4" t="n">
         <v>9</v>
       </c>
-      <c r="E12" t="n">
+      <c r="E17" s="4" t="n">
         <v>1960</v>
       </c>
-      <c r="F12" t="n">
+      <c r="F17" s="4" t="n">
         <v>2026</v>
       </c>
-      <c r="G12" t="n">
+      <c r="G17" s="4" t="n">
         <v>2025</v>
       </c>
-      <c r="H12" t="inlineStr">
+      <c r="H17" s="4" t="inlineStr">
         <is>
           <t>assets/data/world-bank/csv/ove_banco_mundial_venezuela_sector_externo.csv</t>
         </is>
       </c>
-      <c r="I12" t="inlineStr">
+      <c r="I17" s="4" t="inlineStr">
         <is>
           <t>assets/data/world-bank/json/ove_banco_mundial_venezuela_sector_externo.json</t>
         </is>
       </c>
-      <c r="J12" t="inlineStr">
+      <c r="J17" s="4" t="inlineStr">
         <is>
           <t>assets/data/world-bank/excel/ove_banco_mundial_venezuela_sector_externo.xlsx</t>
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
         <is>
           <t>Sector público e instituciones</t>
         </is>
       </c>
-      <c r="B13" t="inlineStr">
+      <c r="B18" s="4" t="inlineStr">
         <is>
           <t>sector_publico_e_instituciones</t>
         </is>
       </c>
-      <c r="C13" t="n">
+      <c r="C18" s="4" t="n">
         <v>268</v>
       </c>
-      <c r="D13" t="n">
+      <c r="D18" s="4" t="n">
         <v>4</v>
       </c>
-      <c r="E13" t="n">
+      <c r="E18" s="4" t="n">
         <v>1960</v>
       </c>
-      <c r="F13" t="n">
+      <c r="F18" s="4" t="n">
         <v>2026</v>
       </c>
-      <c r="H13" t="inlineStr">
+      <c r="G18" s="4" t="n"/>
+      <c r="H18" s="4" t="inlineStr">
         <is>
           <t>assets/data/world-bank/csv/ove_banco_mundial_venezuela_sector_publico_e_instituciones.csv</t>
         </is>
       </c>
-      <c r="I13" t="inlineStr">
+      <c r="I18" s="4" t="inlineStr">
         <is>
           <t>assets/data/world-bank/json/ove_banco_mundial_venezuela_sector_publico_e_instituciones.json</t>
         </is>
       </c>
-      <c r="J13" t="inlineStr">
+      <c r="J18" s="4" t="inlineStr">
         <is>
           <t>assets/data/world-bank/excel/ove_banco_mundial_venezuela_sector_publico_e_instituciones.xlsx</t>
         </is>
@@ -971,5 +1028,120 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D12"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="24" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="28" customHeight="1">
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Metadatos</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="22" customHeight="1">
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>Catálogo Banco Mundial</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="18" customHeight="1"/>
+    <row r="4" ht="16" customHeight="1"/>
+    <row r="5" ht="8" customHeight="1"/>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>Campo</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>Valor</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="6" t="inlineStr">
+        <is>
+          <t>Organización</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>Observatorio Venezolano de Economía</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="6" t="inlineStr">
+        <is>
+          <t>Dataset</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t>Banco Mundial - Venezuela</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="6" t="inlineStr">
+        <is>
+          <t>Fecha generación</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="6" t="inlineStr">
+        <is>
+          <t>Número de áreas</t>
+        </is>
+      </c>
+      <c r="B10" s="4" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="6" t="inlineStr">
+        <is>
+          <t>Número de indicadores</t>
+        </is>
+      </c>
+      <c r="B11" s="4" t="n">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="6" t="inlineStr">
+        <is>
+          <t>Número de registros</t>
+        </is>
+      </c>
+      <c r="B12" s="4" t="n">
+        <v>5249</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>